<commit_message>
Add cards-contributor, tabs-adventure blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 50
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-28T09:28:50.089Z</t>
+    <t>2026-09-28T11:45:07.211Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -73,7 +73,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-09-28T10:58:45.275Z</t>
+    <t>2026-09-28T11:46:15.035Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -82,6 +82,48 @@
     <t>https://wknd.site/us/en/about-us.html</t>
   </si>
   <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>["hero-teaser","cards-filter"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>adventures-2</t>
+  </si>
+  <si>
+    <t>2026-09-28T11:10:15.306Z</t>
+  </si>
+  <si>
+    <t>Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faqs</t>
+  </si>
+  <si>
+    <t>2026-09-28T11:20:42.398Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
@@ -91,7 +133,7 @@
     <t>us/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-28T10:58:50.464Z</t>
+    <t>2026-09-28T11:46:20.281Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -112,7 +154,7 @@
     <t>adventures</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:21.395Z</t>
+    <t>2026-09-28T11:45:12.786Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -127,7 +169,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:26.126Z</t>
+    <t>2026-09-28T11:45:19.523Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -142,7 +184,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:30.779Z</t>
+    <t>2026-09-28T11:45:25.683Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -157,7 +199,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:36.514Z</t>
+    <t>2026-09-28T11:45:31.060Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -172,7 +214,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:42.483Z</t>
+    <t>2026-09-28T11:45:35.242Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -187,7 +229,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-28T10:14:46.813Z</t>
+    <t>2026-09-28T11:45:40.829Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -208,7 +250,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-09-28T10:35:27.160Z</t>
+    <t>2026-09-28T11:45:47.049Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -223,7 +265,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-28T10:35:32.312Z</t>
+    <t>2026-09-28T11:45:52.758Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -238,7 +280,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-28T10:35:36.546Z</t>
+    <t>2026-09-28T11:45:58.149Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -253,7 +295,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-28T10:35:42.611Z</t>
+    <t>2026-09-28T11:46:04.144Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -268,7 +310,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-28T10:35:47.055Z</t>
+    <t>2026-09-28T11:46:08.760Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -663,12 +705,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="43" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
@@ -766,302 +808,354 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
         <v>46</v>
       </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>32</v>
-      </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H10" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
         <v>78</v>
       </c>
-      <c r="B14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>64</v>
-      </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G14" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G15" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H15" t="s">
-        <v>87</v>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>78</v>
+      </c>
+      <c r="F16" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" t="s">
+        <v>99</v>
+      </c>
+      <c r="G17" t="s">
+        <v>100</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 14 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 52
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-28T13:19:15.535Z</t>
+    <t>2026-09-28T13:43:22.838Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -73,7 +73,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-09-28T13:21:22.430Z</t>
+    <t>2026-09-28T13:43:41.779Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -94,7 +94,7 @@
     <t>adventures-2</t>
   </si>
   <si>
-    <t>2026-09-28T11:46:27.037Z</t>
+    <t>2026-09-28T13:43:32.607Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -115,7 +115,7 @@
     <t>faqs</t>
   </si>
   <si>
-    <t>2026-09-28T11:46:32.982Z</t>
+    <t>2026-09-28T13:21:47.653Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -133,7 +133,7 @@
     <t>us/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-28T13:21:28.943Z</t>
+    <t>2026-09-28T13:43:46.387Z</t>
   </si>
   <si>
     <t>Magazine</t>

</xml_diff>